<commit_message>
chore(release): publication-ready repository cleanup and baseline freeze v1.3.1-FREEZE
</commit_message>
<xml_diff>
--- a/results/reports/decision_report.xlsx
+++ b/results/reports/decision_report.xlsx
@@ -450,7 +450,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0.7775821475801472</t>
+          <t>0.7363379273379228</t>
         </is>
       </c>
     </row>
@@ -462,7 +462,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.336</t>
+          <t>0.432</t>
         </is>
       </c>
     </row>
@@ -474,7 +474,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Low Confidence (P(top-1) &lt; 0.40)</t>
+          <t>Moderate Confidence (0.40 &lt;= P(top-1) &lt; 0.70)</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>334.5</t>
+          <t>335.0</t>
         </is>
       </c>
     </row>
@@ -498,7 +498,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Miscible (Below Critical chi_c = 2.12)</t>
+          <t>Miscible (Below Critical chi_c = 0.56)</t>
         </is>
       </c>
     </row>
@@ -510,7 +510,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -522,7 +522,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0.45714285714285724</t>
+          <t>0.0</t>
         </is>
       </c>
     </row>
@@ -537,7 +537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -571,10 +571,15 @@
           <t>topsis_rank</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>polymer_name</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -583,47 +588,57 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>POL-005-2026</t>
+          <t>SOLUPLUS</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.20132439972428</v>
+        <v>0.3235034398880975</v>
       </c>
       <c r="E2" t="n">
-        <v>0.7038385516032278</v>
+        <v>0.9034589237989848</v>
       </c>
       <c r="F2" t="n">
-        <v>0.7775821475801472</v>
+        <v>0.7363379273379228</v>
       </c>
       <c r="G2" t="n">
         <v>1</v>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Soluplus</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>POL-003-2026</t>
+          <t>POL-006-2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>POL-003-2026</t>
+          <t>HPMC_E5</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.2278800758598495</v>
+        <v>0.3115688695726735</v>
       </c>
       <c r="E3" t="n">
-        <v>0.6311018931095516</v>
+        <v>0.6746059747360333</v>
       </c>
       <c r="F3" t="n">
-        <v>0.7347091276744051</v>
+        <v>0.6840632557494626</v>
       </c>
       <c r="G3" t="n">
         <v>2</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Hydroxypropyl Methylcellulose E5</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -637,20 +652,25 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>POL-002-2026</t>
+          <t>PVP_VA_64</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.305701575106238</v>
+        <v>0.484852953730242</v>
       </c>
       <c r="E4" t="n">
-        <v>0.5177985760197286</v>
+        <v>0.494612513147383</v>
       </c>
       <c r="F4" t="n">
-        <v>0.6287777546995539</v>
+        <v>0.5049820844874975</v>
       </c>
       <c r="G4" t="n">
         <v>3</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>PVP-Vinyl Acetate 64</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -664,74 +684,57 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>POL-001-2026</t>
+          <t>PVP_K30</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.5400380995973019</v>
+        <v>0.5774374955017395</v>
       </c>
       <c r="E5" t="n">
-        <v>0.4014348914080261</v>
+        <v>0.459099433308197</v>
       </c>
       <c r="F5" t="n">
-        <v>0.4263902366220448</v>
+        <v>0.4429166202841378</v>
       </c>
       <c r="G5" t="n">
         <v>4</v>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Polyvinylpyrrolidone K30</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>POL-006-2026</t>
+          <t>POL-007-2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>POL-006-2026</t>
+          <t>EDR_EPO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.6083843485113785</v>
+        <v>0.959686095962783</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2034565733577816</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0.2506113794921163</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
         <v>5</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>POL-004-2026</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>POL-004-2026</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>0.7205586217520539</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0.1464470781172874</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0.16891132104363</v>
-      </c>
-      <c r="G7" t="n">
-        <v>6</v>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Eudragit E PO</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(freeze): establish v1.4.0-CORRECTED-FREEZE baseline with verified Flory-Huggins and Tm bugfixes
</commit_message>
<xml_diff>
--- a/results/reports/decision_report.xlsx
+++ b/results/reports/decision_report.xlsx
@@ -438,7 +438,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Soluplus</t>
+          <t>Hydroxypropyl Methylcellulose E5</t>
         </is>
       </c>
     </row>
@@ -450,7 +450,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0.7363379273379228</t>
+          <t>0.8359112438004079</t>
         </is>
       </c>
     </row>
@@ -462,7 +462,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.432</t>
+          <t>0.424</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>335.0</t>
+          <t>393.8</t>
         </is>
       </c>
     </row>
@@ -498,7 +498,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Miscible (Below Critical chi_c = 0.56)</t>
+          <t>Miscible (Below Critical chi_c = 0.64)</t>
         </is>
       </c>
     </row>
@@ -522,7 +522,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>-0.3643060444313498</t>
         </is>
       </c>
     </row>
@@ -579,129 +579,129 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>POL-005-2026</t>
+          <t>POL-006-2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SOLUPLUS</t>
+          <t>HPMC_E5</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.3235034398880975</v>
+        <v>0.1561784025045568</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9034589237989848</v>
+        <v>0.7956138233721912</v>
       </c>
       <c r="F2" t="n">
-        <v>0.7363379273379228</v>
+        <v>0.8359112438004079</v>
       </c>
       <c r="G2" t="n">
         <v>1</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Soluplus</t>
+          <t>Hydroxypropyl Methylcellulose E5</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>POL-006-2026</t>
+          <t>POL-005-2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>HPMC_E5</t>
+          <t>SOLUPLUS</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.3115688695726735</v>
+        <v>0.3822661559243256</v>
       </c>
       <c r="E3" t="n">
-        <v>0.6746059747360333</v>
+        <v>0.8683684982468969</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6840632557494626</v>
+        <v>0.6943422648258153</v>
       </c>
       <c r="G3" t="n">
         <v>2</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Hydroxypropyl Methylcellulose E5</t>
+          <t>Soluplus</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>POL-002-2026</t>
+          <t>POL-001-2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PVP_VA_64</t>
+          <t>PVP_K30</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.484852953730242</v>
+        <v>0.4592717296104521</v>
       </c>
       <c r="E4" t="n">
-        <v>0.494612513147383</v>
+        <v>0.5598996160687572</v>
       </c>
       <c r="F4" t="n">
-        <v>0.5049820844874975</v>
+        <v>0.5493675017870735</v>
       </c>
       <c r="G4" t="n">
         <v>3</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>PVP-Vinyl Acetate 64</t>
+          <t>Polyvinylpyrrolidone K30</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>POL-001-2026</t>
+          <t>POL-002-2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>PVP_K30</t>
+          <t>PVP_VA_64</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.5774374955017395</v>
+        <v>0.5062927873276735</v>
       </c>
       <c r="E5" t="n">
-        <v>0.459099433308197</v>
+        <v>0.4494387963264038</v>
       </c>
       <c r="F5" t="n">
-        <v>0.4429166202841378</v>
+        <v>0.470256297911649</v>
       </c>
       <c r="G5" t="n">
         <v>4</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Polyvinylpyrrolidone K30</t>
+          <t>PVP-Vinyl Acetate 64</t>
         </is>
       </c>
     </row>
@@ -720,13 +720,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.959686095962783</v>
+        <v>0.9158716125052487</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>0.09113566654646343</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>0.09050149730028258</v>
       </c>
       <c r="G6" t="n">
         <v>5</v>

</xml_diff>

<commit_message>
feat(release): freeze v1.5.0-FOUR-CRITERION-FREEZE baseline and release PharmaPolySCOPE
- Freeze authoritative v1.5.0 four-criterion computational baseline (s_HSP, s_chi, s_desc, s_GT)
- Permanently isolate literature score (s_lit) to provenance metadata
- Establish Policy A fixed-subspace Monte Carlo uncertainty quantification (N=10,000, seed=42)
- Confirm deterministic ranking: HPMC E5 (Rank 1, CL=0.8359, P(top-1)=75.54%)
- Integrate official PharmaPolySCOPE branding, Lattice Lens logo assets, and developer attribution
- Implement 14-page dynamic PDF technical report generator with full provenance snapshot
- Synchronize complete documentation suite and machine-readable baseline manifest
- Validate complete 76/76 automated test suite and 0-error frontend production build
</commit_message>
<xml_diff>
--- a/results/reports/decision_report.xlsx
+++ b/results/reports/decision_report.xlsx
@@ -462,7 +462,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.424</t>
+          <t>0.7554</t>
         </is>
       </c>
     </row>
@@ -474,7 +474,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Moderate Confidence (0.40 &lt;= P(top-1) &lt; 0.70)</t>
+          <t>High Confidence (P(top-1) &gt;= 0.70)</t>
         </is>
       </c>
     </row>
@@ -498,7 +498,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Miscible (Below Critical chi_c = 0.64)</t>
+          <t>Phase-boundary diagnostic favorable (chi = 0.260 &lt; critical chi_c = 0.640)</t>
         </is>
       </c>
     </row>

</xml_diff>